<commit_message>
Commit for 11 October 2026
</commit_message>
<xml_diff>
--- a/12600351.xlsx
+++ b/12600351.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sage/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6F2A447-7D23-8D4D-B68D-E6D6EF375724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5CF219-4375-8B4A-B796-F7FE744C2450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="100">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -334,6 +334,9 @@
   </si>
   <si>
     <t>Learned Kadane's Algorithm and Completed Minor Project of Python.</t>
+  </si>
+  <si>
+    <t>Solved Analytical Exercise on HitBullsEye.</t>
   </si>
 </sst>
 </file>
@@ -3118,27 +3121,51 @@
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A49" s="12"/>
-      <c r="B49" s="13"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="13"/>
-      <c r="E49" s="13"/>
-      <c r="F49" s="13"/>
-      <c r="G49" s="13"/>
-      <c r="H49" s="13"/>
-      <c r="I49" s="14" t="str">
+    <row r="49" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+      <c r="A49" s="12">
+        <v>46306</v>
+      </c>
+      <c r="B49" s="13">
+        <v>460</v>
+      </c>
+      <c r="C49" s="13">
+        <v>0</v>
+      </c>
+      <c r="D49" s="13">
+        <v>400</v>
+      </c>
+      <c r="E49" s="13">
+        <v>60</v>
+      </c>
+      <c r="F49" s="13">
+        <v>0</v>
+      </c>
+      <c r="G49" s="13">
+        <v>0</v>
+      </c>
+      <c r="H49" s="13">
+        <v>400</v>
+      </c>
+      <c r="I49" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="14" t="str">
+        <v>1320</v>
+      </c>
+      <c r="J49" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K49" s="15"/>
-      <c r="L49" s="15"/>
-      <c r="M49" s="15"/>
-      <c r="N49" s="16"/>
+        <v>120</v>
+      </c>
+      <c r="K49" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="L49" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="M49" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="N49" s="16" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="12"/>

</xml_diff>